<commit_message>
Update Philly BYOB Restaurant_with_websites_merged.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant_with_websites_merged.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant_with_websites_merged.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0972039C-DF36-4EBB-80B7-4B19A7AF5822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E61A712-6B67-4D64-B92F-C88BA2B15024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="472">
   <si>
     <t>WP_Post_ID</t>
   </si>
@@ -1238,6 +1251,204 @@
   </si>
   <si>
     <t>Ristorante Aroma</t>
+  </si>
+  <si>
+    <t>Alyan’s Middle Eastern &amp; Mediterranean Restaurant</t>
+  </si>
+  <si>
+    <t>603 S 4th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 922-3553  </t>
+  </si>
+  <si>
+    <t>Apricot Stone</t>
+  </si>
+  <si>
+    <t>428 W Girard Ave, Philadelphia, PA 19123 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(267) 606-6596  </t>
+  </si>
+  <si>
+    <t>1247 S 13th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 465-2200  </t>
+  </si>
+  <si>
+    <t>Casablanca Mediterranean Grill</t>
+  </si>
+  <si>
+    <t>947 Federal St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(267) 324-5165  </t>
+  </si>
+  <si>
+    <t>Chabba Thai bistro</t>
+  </si>
+  <si>
+    <t>4343 Main St, Philadelphia, PA 19127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 483-1979  </t>
+  </si>
+  <si>
+    <t>Fiorino</t>
+  </si>
+  <si>
+    <t>3572 Indian Queen Ln, Philadelphia, PA 19129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 843-1500  </t>
+  </si>
+  <si>
+    <t>Han dynasty (manayunk)</t>
+  </si>
+  <si>
+    <t>4356 Main St, Philadelphia, PA 19127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 508-2066  </t>
+  </si>
+  <si>
+    <t>June BYOB</t>
+  </si>
+  <si>
+    <t> 690 Haddon Ave, Collingswood, NJ 08108 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(856) 240-7041  </t>
+  </si>
+  <si>
+    <t>Kung Fu Hot Pot</t>
+  </si>
+  <si>
+    <t>1008 Cherry St 3rd floor, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 606-1899  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(267) 928-3262  </t>
+  </si>
+  <si>
+    <t>Sakartvelo</t>
+  </si>
+  <si>
+    <t>705 Chestnut St, Philadelphia, PA 19106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(267) 319-1631  </t>
+  </si>
+  <si>
+    <t>Scampi</t>
+  </si>
+  <si>
+    <t> 617 S 3rd St, Philadelphia, PA 19147 </t>
+  </si>
+  <si>
+    <t>Vientiane Bistro</t>
+  </si>
+  <si>
+    <t>2537 Kensington Ave, Philadelphia, PA 19125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(267) 703-8199  </t>
+  </si>
+  <si>
+    <t>White yak</t>
+  </si>
+  <si>
+    <t> 6118 Ridge Ave, Philadelphia, PA 19128 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 483-0764  </t>
+  </si>
+  <si>
+    <t>Yamitsuki</t>
+  </si>
+  <si>
+    <t>1028 Arch St , Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(215) 629-3888  </t>
+  </si>
+  <si>
+    <t>Yanako restaurant</t>
+  </si>
+  <si>
+    <t>4345 Main St, Philadelphia, PA 19127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(267) 297-8151  </t>
+  </si>
+  <si>
+    <t>Zeppoli</t>
+  </si>
+  <si>
+    <t>618 Collings Ave, Collingswood NJ 08107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(856) 854-2670  </t>
+  </si>
+  <si>
+    <t>https://www.scampiphilly.com/menu</t>
+  </si>
+  <si>
+    <t>http://www.junebyob.com/</t>
+  </si>
+  <si>
+    <t>http://www.zeppolirestaurant.com/</t>
+  </si>
+  <si>
+    <t>http://www.casablanca-grill.com/</t>
+  </si>
+  <si>
+    <t>https://www.fiorino.us/</t>
+  </si>
+  <si>
+    <t>http://www.handynasty.net/</t>
+  </si>
+  <si>
+    <t>https://whiteyakrestaurant.com/?utm_source=google</t>
+  </si>
+  <si>
+    <t>https://www.vientianebistro.com/</t>
+  </si>
+  <si>
+    <t>https://theyanako.com/</t>
+  </si>
+  <si>
+    <t>https://chabaathai.com/</t>
+  </si>
+  <si>
+    <t>http://www.apricotstonephilly.com/</t>
+  </si>
+  <si>
+    <t>https://sakartvelopa.com/</t>
+  </si>
+  <si>
+    <t>https://yamitsuki1028.wixsite.com/yamitsukiramen</t>
+  </si>
+  <si>
+    <t>info@junebyob.com</t>
+  </si>
+  <si>
+    <t>casablancamg947@gmail.com</t>
+  </si>
+  <si>
+    <t>treley@whiteyakrestaurant.com</t>
+  </si>
+  <si>
+    <t>astigma@astigmatic.com</t>
+  </si>
+  <si>
+    <t>info@apricotstonephilly.com</t>
+  </si>
+  <si>
+    <t>yamitsuki1028@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1245,7 +1456,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="179" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -1310,7 +1521,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1613,10 +1824,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S73"/>
+  <dimension ref="A1:S90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="21.125" customWidth="1"/>
+    <col min="9" max="9" width="11.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.3">
@@ -1703,7 +1916,7 @@
       <c r="H2">
         <v>-75.1753073</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J2" t="s">
@@ -1735,7 +1948,7 @@
       <c r="H3">
         <v>-75.152359599999997</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1764,7 +1977,7 @@
       <c r="H4">
         <v>-75.179640800000001</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1790,7 +2003,7 @@
       <c r="H5">
         <v>-75.170259099999996</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J5" t="s">
@@ -1822,7 +2035,7 @@
       <c r="H6">
         <v>-75.165249199999991</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J6" t="s">
@@ -1857,7 +2070,7 @@
       <c r="H7">
         <v>-75.144517199999996</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J7" t="s">
@@ -1889,7 +2102,7 @@
       <c r="H8">
         <v>-75.141018599999995</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J8" t="s">
@@ -1921,7 +2134,7 @@
       <c r="H9">
         <v>-75.161606300000003</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J9" t="s">
@@ -1950,7 +2163,7 @@
       <c r="H10">
         <v>-75.129705099999995</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J10" t="s">
@@ -1982,7 +2195,7 @@
       <c r="H11">
         <v>-75.164066699999992</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2011,7 +2224,7 @@
       <c r="H12">
         <v>-75.164232699999999</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2040,7 +2253,7 @@
       <c r="H13">
         <v>-75.144519399999993</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2069,7 +2282,7 @@
       <c r="H14">
         <v>-75.140985200000003</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J14" t="s">
@@ -2098,7 +2311,7 @@
       <c r="H15">
         <v>-75.180016899999998</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J15" t="s">
@@ -2130,7 +2343,7 @@
       <c r="H16">
         <v>-75.170737899999992</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2156,7 +2369,7 @@
       <c r="H17">
         <v>-75.160454999999999</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2185,7 +2398,7 @@
       <c r="H18">
         <v>-75.160108000000008</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I18" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2211,7 +2424,7 @@
       <c r="H19">
         <v>-75.134557399999991</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2240,7 +2453,7 @@
       <c r="H20">
         <v>-75.146249400000002</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2269,7 +2482,7 @@
       <c r="H21">
         <v>-75.167785299999991</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2295,7 +2508,7 @@
       <c r="H22">
         <v>-75.171386099999992</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2324,7 +2537,7 @@
       <c r="H23">
         <v>-75.171194099999994</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2350,7 +2563,7 @@
       <c r="H24">
         <v>-75.152963700000001</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J24" t="s">
@@ -2382,7 +2595,7 @@
       <c r="H25">
         <v>-75.173786499999991</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J25" t="s">
@@ -2414,7 +2627,7 @@
       <c r="H26">
         <v>-75.157853799999998</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2443,7 +2656,7 @@
       <c r="H27">
         <v>-75.174123500000007</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J27" t="s">
@@ -2475,7 +2688,7 @@
       <c r="H28">
         <v>-75.161768199999997</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I28" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J28" t="s">
@@ -2510,7 +2723,7 @@
       <c r="H29">
         <v>-75.160984799999994</v>
       </c>
-      <c r="I29" t="s">
+      <c r="I29" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2539,7 +2752,7 @@
       <c r="H30">
         <v>-75.170019699999997</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I30" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2568,7 +2781,7 @@
       <c r="H31">
         <v>-75.144386900000001</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J31" t="s">
@@ -2600,7 +2813,7 @@
       <c r="H32">
         <v>-75.156515900000002</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J32" t="s">
@@ -2632,7 +2845,7 @@
       <c r="H33">
         <v>-75.140709299999997</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J33" t="s">
@@ -2661,7 +2874,7 @@
       <c r="H34">
         <v>-75.175115599999998</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I34" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2690,7 +2903,7 @@
       <c r="H35">
         <v>-75.167463699999999</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2716,7 +2929,7 @@
       <c r="H36">
         <v>-75.16734799999999</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2745,7 +2958,7 @@
       <c r="H37">
         <v>-75.171119699999991</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2774,7 +2987,7 @@
       <c r="H38">
         <v>-75.174716699999991</v>
       </c>
-      <c r="I38" t="s">
+      <c r="I38" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J38" t="s">
@@ -2806,7 +3019,7 @@
       <c r="H39">
         <v>-75.155556500000003</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I39" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2835,7 +3048,7 @@
       <c r="H40">
         <v>-75.185306799999992</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I40" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J40" t="s">
@@ -2867,7 +3080,7 @@
       <c r="H41">
         <v>-75.177968399999997</v>
       </c>
-      <c r="I41" t="s">
+      <c r="I41" s="2" t="s">
         <v>24</v>
       </c>
       <c r="J41" t="s">
@@ -2899,7 +3112,7 @@
       <c r="H42">
         <v>-75.174830900000003</v>
       </c>
-      <c r="I42" t="s">
+      <c r="I42" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2928,7 +3141,7 @@
       <c r="H43">
         <v>-75.217944799999998</v>
       </c>
-      <c r="I43" t="s">
+      <c r="I43" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2957,7 +3170,7 @@
       <c r="H44">
         <v>-75.149544399999996</v>
       </c>
-      <c r="I44" t="s">
+      <c r="I44" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -2983,7 +3196,7 @@
       <c r="H45">
         <v>-75.050069499999992</v>
       </c>
-      <c r="I45" t="s">
+      <c r="I45" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3009,7 +3222,7 @@
       <c r="H46">
         <v>-75.154025899999993</v>
       </c>
-      <c r="I46" t="s">
+      <c r="I46" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J46" t="s">
@@ -3041,7 +3254,7 @@
       <c r="H47">
         <v>-75.149088399999997</v>
       </c>
-      <c r="I47" t="s">
+      <c r="I47" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3067,7 +3280,7 @@
       <c r="H48">
         <v>-75.156259599999998</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I48" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3096,7 +3309,7 @@
       <c r="H49">
         <v>-75.178519699999995</v>
       </c>
-      <c r="I49" t="s">
+      <c r="I49" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3125,7 +3338,7 @@
       <c r="H50">
         <v>-75.150354600000014</v>
       </c>
-      <c r="I50" t="s">
+      <c r="I50" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J50" t="s">
@@ -3160,7 +3373,7 @@
       <c r="H51">
         <v>-75.034327399999995</v>
       </c>
-      <c r="I51" t="s">
+      <c r="I51" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3186,7 +3399,7 @@
       <c r="H52">
         <v>-75.171258600000002</v>
       </c>
-      <c r="I52" t="s">
+      <c r="I52" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3209,7 +3422,7 @@
       <c r="H53">
         <v>-75.173383200000004</v>
       </c>
-      <c r="I53" t="s">
+      <c r="I53" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3238,7 +3451,7 @@
       <c r="H54">
         <v>-75.157960899999992</v>
       </c>
-      <c r="I54" t="s">
+      <c r="I54" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J54" t="s">
@@ -3273,7 +3486,7 @@
       <c r="H55">
         <v>-75.153989299999992</v>
       </c>
-      <c r="I55" t="s">
+      <c r="I55" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3302,7 +3515,7 @@
       <c r="H56">
         <v>-75.16970049999999</v>
       </c>
-      <c r="I56" t="s">
+      <c r="I56" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J56" t="s">
@@ -3331,7 +3544,7 @@
       <c r="H57">
         <v>-75.169153299999991</v>
       </c>
-      <c r="I57" t="s">
+      <c r="I57" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3360,7 +3573,7 @@
       <c r="H58">
         <v>-75.190036300000003</v>
       </c>
-      <c r="I58" t="s">
+      <c r="I58" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J58" t="s">
@@ -3398,7 +3611,7 @@
       <c r="H59">
         <v>-75.163266499999992</v>
       </c>
-      <c r="I59" t="s">
+      <c r="I59" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J59" t="s">
@@ -3430,7 +3643,7 @@
       <c r="H60">
         <v>-75.157535600000003</v>
       </c>
-      <c r="I60" t="s">
+      <c r="I60" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3459,7 +3672,7 @@
       <c r="H61">
         <v>-75.172149099999999</v>
       </c>
-      <c r="I61" t="s">
+      <c r="I61" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J61" t="s">
@@ -3491,7 +3704,7 @@
       <c r="H62">
         <v>-75.102839599999996</v>
       </c>
-      <c r="I62" t="s">
+      <c r="I62" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J62" t="s">
@@ -3523,7 +3736,7 @@
       <c r="H63">
         <v>-75.146044199999992</v>
       </c>
-      <c r="I63" t="s">
+      <c r="I63" s="2" t="s">
         <v>246</v>
       </c>
     </row>
@@ -3552,7 +3765,7 @@
       <c r="H64">
         <v>-75.159783899999994</v>
       </c>
-      <c r="I64" t="s">
+      <c r="I64" s="2" t="s">
         <v>246</v>
       </c>
       <c r="J64" t="s">
@@ -3562,7 +3775,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>1747</v>
       </c>
@@ -3587,11 +3800,11 @@
       <c r="H65">
         <v>-75.113133699999992</v>
       </c>
-      <c r="I65" t="s">
+      <c r="I65" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>1748</v>
       </c>
@@ -3616,11 +3829,11 @@
       <c r="H66">
         <v>-75.147412399999993</v>
       </c>
-      <c r="I66" t="s">
+      <c r="I66" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>1749</v>
       </c>
@@ -3645,11 +3858,11 @@
       <c r="H67">
         <v>-75.174111199999999</v>
       </c>
-      <c r="I67" t="s">
+      <c r="I67" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>1750</v>
       </c>
@@ -3674,11 +3887,11 @@
       <c r="H68">
         <v>-75.160342099999994</v>
       </c>
-      <c r="I68" t="s">
+      <c r="I68" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>1754</v>
       </c>
@@ -3703,14 +3916,14 @@
       <c r="H69">
         <v>-75.177395099999998</v>
       </c>
-      <c r="I69" t="s">
+      <c r="I69" s="2" t="s">
         <v>380</v>
       </c>
       <c r="J69" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>1755</v>
       </c>
@@ -3732,14 +3945,14 @@
       <c r="H70">
         <v>-75.182546800000011</v>
       </c>
-      <c r="I70" t="s">
+      <c r="I70" s="2" t="s">
         <v>380</v>
       </c>
       <c r="J70" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>1756</v>
       </c>
@@ -3764,14 +3977,14 @@
       <c r="H71">
         <v>-75.129835499999999</v>
       </c>
-      <c r="I71" t="s">
+      <c r="I71" s="2" t="s">
         <v>380</v>
       </c>
       <c r="J71" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>1757</v>
       </c>
@@ -3796,14 +4009,14 @@
       <c r="H72">
         <v>-75.160762800000001</v>
       </c>
-      <c r="I72" t="s">
+      <c r="I72" s="2" t="s">
         <v>398</v>
       </c>
       <c r="J72" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>1402</v>
       </c>
@@ -3830,6 +4043,463 @@
       </c>
       <c r="I73" s="2">
         <v>45985</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>1408</v>
+      </c>
+      <c r="B74" t="s">
+        <v>406</v>
+      </c>
+      <c r="C74" t="s">
+        <v>407</v>
+      </c>
+      <c r="D74" t="s">
+        <v>408</v>
+      </c>
+      <c r="G74">
+        <v>39.941414799999997</v>
+      </c>
+      <c r="H74">
+        <v>-75.149054199999995</v>
+      </c>
+      <c r="I74" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>1389</v>
+      </c>
+      <c r="B75" t="s">
+        <v>409</v>
+      </c>
+      <c r="C75" t="s">
+        <v>410</v>
+      </c>
+      <c r="D75" t="s">
+        <v>411</v>
+      </c>
+      <c r="E75" t="s">
+        <v>463</v>
+      </c>
+      <c r="G75">
+        <v>39.969888599999997</v>
+      </c>
+      <c r="H75">
+        <v>-75.144038499999994</v>
+      </c>
+      <c r="I75" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J75" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>1374</v>
+      </c>
+      <c r="B76" t="s">
+        <v>41</v>
+      </c>
+      <c r="C76" t="s">
+        <v>412</v>
+      </c>
+      <c r="D76" t="s">
+        <v>413</v>
+      </c>
+      <c r="E76" t="s">
+        <v>44</v>
+      </c>
+      <c r="G76">
+        <v>39.933934299999997</v>
+      </c>
+      <c r="H76">
+        <v>-75.165249199999991</v>
+      </c>
+      <c r="I76" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J76" t="s">
+        <v>47</v>
+      </c>
+      <c r="K76" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>1407</v>
+      </c>
+      <c r="B77" t="s">
+        <v>414</v>
+      </c>
+      <c r="C77" t="s">
+        <v>415</v>
+      </c>
+      <c r="D77" t="s">
+        <v>416</v>
+      </c>
+      <c r="E77" t="s">
+        <v>456</v>
+      </c>
+      <c r="G77">
+        <v>39.9346672</v>
+      </c>
+      <c r="H77">
+        <v>-75.160286099999993</v>
+      </c>
+      <c r="I77" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J77" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>1398</v>
+      </c>
+      <c r="B78" t="s">
+        <v>417</v>
+      </c>
+      <c r="C78" t="s">
+        <v>418</v>
+      </c>
+      <c r="D78" t="s">
+        <v>419</v>
+      </c>
+      <c r="E78" t="s">
+        <v>462</v>
+      </c>
+      <c r="G78">
+        <v>40.025693400000002</v>
+      </c>
+      <c r="H78">
+        <v>-75.2233971</v>
+      </c>
+      <c r="I78" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>1401</v>
+      </c>
+      <c r="B79" t="s">
+        <v>420</v>
+      </c>
+      <c r="C79" t="s">
+        <v>421</v>
+      </c>
+      <c r="D79" t="s">
+        <v>422</v>
+      </c>
+      <c r="E79" t="s">
+        <v>457</v>
+      </c>
+      <c r="G79">
+        <v>40.009791999999997</v>
+      </c>
+      <c r="H79">
+        <v>-75.190426099999996</v>
+      </c>
+      <c r="I79" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>1404</v>
+      </c>
+      <c r="B80" t="s">
+        <v>423</v>
+      </c>
+      <c r="C80" t="s">
+        <v>424</v>
+      </c>
+      <c r="D80" t="s">
+        <v>425</v>
+      </c>
+      <c r="E80" t="s">
+        <v>458</v>
+      </c>
+      <c r="G80">
+        <v>40.025373700000003</v>
+      </c>
+      <c r="H80">
+        <v>-75.223862799999992</v>
+      </c>
+      <c r="I80" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>1410</v>
+      </c>
+      <c r="B81" t="s">
+        <v>426</v>
+      </c>
+      <c r="C81" t="s">
+        <v>427</v>
+      </c>
+      <c r="D81" t="s">
+        <v>428</v>
+      </c>
+      <c r="E81" t="s">
+        <v>454</v>
+      </c>
+      <c r="G81">
+        <v>39.916215800000003</v>
+      </c>
+      <c r="H81">
+        <v>-75.069438599999998</v>
+      </c>
+      <c r="I81" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J81" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>1417</v>
+      </c>
+      <c r="B82" t="s">
+        <v>429</v>
+      </c>
+      <c r="C82" t="s">
+        <v>430</v>
+      </c>
+      <c r="D82" t="s">
+        <v>431</v>
+      </c>
+      <c r="G82">
+        <v>39.954462199999988</v>
+      </c>
+      <c r="H82">
+        <v>-75.156541500000003</v>
+      </c>
+      <c r="I82" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>1377</v>
+      </c>
+      <c r="B83" t="s">
+        <v>114</v>
+      </c>
+      <c r="C83" t="s">
+        <v>115</v>
+      </c>
+      <c r="D83" t="s">
+        <v>432</v>
+      </c>
+      <c r="E83" t="s">
+        <v>117</v>
+      </c>
+      <c r="G83">
+        <v>39.941107500000001</v>
+      </c>
+      <c r="H83">
+        <v>-75.146249400000002</v>
+      </c>
+      <c r="I83" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>1388</v>
+      </c>
+      <c r="B84" t="s">
+        <v>433</v>
+      </c>
+      <c r="C84" t="s">
+        <v>434</v>
+      </c>
+      <c r="D84" t="s">
+        <v>435</v>
+      </c>
+      <c r="E84" t="s">
+        <v>464</v>
+      </c>
+      <c r="G84">
+        <v>39.949672</v>
+      </c>
+      <c r="H84">
+        <v>-75.152562000000017</v>
+      </c>
+      <c r="I84" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>1412</v>
+      </c>
+      <c r="B85" t="s">
+        <v>436</v>
+      </c>
+      <c r="C85" t="s">
+        <v>437</v>
+      </c>
+      <c r="E85" t="s">
+        <v>453</v>
+      </c>
+      <c r="G85">
+        <v>39.940898199999999</v>
+      </c>
+      <c r="H85">
+        <v>-75.147503599999993</v>
+      </c>
+      <c r="I85" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>1383</v>
+      </c>
+      <c r="B86" t="s">
+        <v>438</v>
+      </c>
+      <c r="C86" t="s">
+        <v>439</v>
+      </c>
+      <c r="D86" t="s">
+        <v>440</v>
+      </c>
+      <c r="E86" t="s">
+        <v>460</v>
+      </c>
+      <c r="G86">
+        <v>39.988109899999998</v>
+      </c>
+      <c r="H86">
+        <v>-75.1282341</v>
+      </c>
+      <c r="I86" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J86" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>1376</v>
+      </c>
+      <c r="B87" t="s">
+        <v>441</v>
+      </c>
+      <c r="C87" t="s">
+        <v>442</v>
+      </c>
+      <c r="D87" t="s">
+        <v>443</v>
+      </c>
+      <c r="E87" t="s">
+        <v>459</v>
+      </c>
+      <c r="G87">
+        <v>40.033780200000002</v>
+      </c>
+      <c r="H87">
+        <v>-75.21579659999999</v>
+      </c>
+      <c r="I87" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J87" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>1387</v>
+      </c>
+      <c r="B88" t="s">
+        <v>444</v>
+      </c>
+      <c r="C88" t="s">
+        <v>445</v>
+      </c>
+      <c r="D88" t="s">
+        <v>446</v>
+      </c>
+      <c r="E88" t="s">
+        <v>465</v>
+      </c>
+      <c r="G88">
+        <v>39.953542300000002</v>
+      </c>
+      <c r="H88">
+        <v>-75.157455200000001</v>
+      </c>
+      <c r="I88" s="2">
+        <v>45987</v>
+      </c>
+      <c r="J88" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>1399</v>
+      </c>
+      <c r="B89" t="s">
+        <v>447</v>
+      </c>
+      <c r="C89" t="s">
+        <v>448</v>
+      </c>
+      <c r="D89" t="s">
+        <v>449</v>
+      </c>
+      <c r="E89" t="s">
+        <v>461</v>
+      </c>
+      <c r="G89">
+        <v>40.025600900000001</v>
+      </c>
+      <c r="H89">
+        <v>-75.2234981</v>
+      </c>
+      <c r="I89" s="2">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>1409</v>
+      </c>
+      <c r="B90" t="s">
+        <v>450</v>
+      </c>
+      <c r="C90" t="s">
+        <v>451</v>
+      </c>
+      <c r="D90" t="s">
+        <v>452</v>
+      </c>
+      <c r="E90" t="s">
+        <v>455</v>
+      </c>
+      <c r="G90">
+        <v>39.910713899999998</v>
+      </c>
+      <c r="H90">
+        <v>-75.084474200000002</v>
+      </c>
+      <c r="I90" s="2">
+        <v>45987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>